<commit_message>
chore: update Тест Еllanse.xlsx with corrections
</commit_message>
<xml_diff>
--- a/Тест Еllanse.xlsx
+++ b/Тест Еllanse.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="22527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\headofmed\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\itd\Desktop\Код\aesthetic_bot\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7445FD8F-99FC-434C-BC2D-673C431F20C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52F67737-5B09-41D1-B34B-E8E7DF667EB0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Інструкція" sheetId="1" r:id="rId1"/>
@@ -182,15 +182,6 @@
     <t>Сферичні,з гладкою поверхнею, 25–50 μm</t>
   </si>
   <si>
-    <t>Мікросфери полікапролактону в Ellansé мають
-оптимальну біосумісність: гладеньку поверхню,
-сферичну форму, розмір 25–50 μm, повну
-біодеградацію з часом.
-→ 'Лікар, ГК вимагає повтор кожні 9–12 місяців. Ellansé — раз на 2–4 роки. Пацієнт витрачає менше в сумі, а клініка отримує більший разовий чек і лояльного клієнта.'
-*Заперечення 'Є постачальник Juvederm':*
-→ 'Juvederm — чудовий ГК-філер для об'єму. Ellansé вирішує інше завдання — омолодження через власний колаген. Вони не замінюють, а доповнюють одне одного.'</t>
-  </si>
-  <si>
     <t>Унікальний процес біодеградації дозволяє
 уникнути вираженого запалення та сприяє
 довготривалій стимуляції колагену І типу</t>
@@ -228,6 +219,185 @@
   </si>
   <si>
     <t>Концентрацією карбоксиметилцелюлози</t>
+  </si>
+  <si>
+    <t>Механізм дії та показання до застосування препарату Ellanse</t>
+  </si>
+  <si>
+    <t>Який механізм дії Ellanse?</t>
+  </si>
+  <si>
+    <t>1 крок: Миттєве відновлення об'єму,  2 крок: стимуляція синтезу власного колагену</t>
+  </si>
+  <si>
+    <t>1 крок:підготовка до синтезу колагену; 2 крок - синтез колагену; 3 крок -розпад колагену</t>
+  </si>
+  <si>
+    <t>1. Крок біоревіталізація; 2-біорепарація; 3- реструктуризація</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 крок відновлення об'єму; 2 крок-біодеградація </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Подвійна дія  Ellanse: 1.МИТТЄВЕ
+ВІДНОВЛЕННЯ ОБ’ЄМУ.Відбувається завдяки карбоксиметилцелюлозі
+Ellansé містить гладкі мікросфери,
+рівномірно розподілені в гелі-носії,
+які заповнюють ділянки шкіри,
+відновлюючи втрачений об’єм. КРОК 2: СТИМУЛЯЦІЯ
+СИНТЕЗУ ВЛАСНОГО
+КОЛАГЕНУ(довгострокова волюмізація-відбуваєтся завдяки полікапролактону):Протягом кількох місяців наявність
+гладких мікросфер посилює
+природний синтез колагену в
+шкірі. Мікросфери біодеградують
+із часом, а колагенові структури
+залишаються
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ellanse показаний 1.Чоловікам та  жінкам старше 18 років
+2.З будь-яким типом старіння
+3.Які хочуть поступових покращень з довгостроковим результатом:
+-Untouched face
+-Відновлення втрачених об’ємів
+-Ліфтингу
+-Зменшення асиметрії
+-Чіткого контуру та овалу  обличчя
+-Покращення пружності та еластичності шкіри
+</t>
+  </si>
+  <si>
+    <t>Що НЕ являється показанням для проведення процедури Ellanse</t>
+  </si>
+  <si>
+    <t>Untouched face</t>
+  </si>
+  <si>
+    <t>Втрата об'єму</t>
+  </si>
+  <si>
+    <t>Зниження пружності шкіри</t>
+  </si>
+  <si>
+    <t>Гіперпігментація</t>
+  </si>
+  <si>
+    <t>Механізм дії та показання до застосування препарату Ellanse,зонивведення</t>
+  </si>
+  <si>
+    <t>Ellanse використовується тільки для корекції наступних зон обличчя:ВЕРХНЯ
+ТРЕТИНА ОБЛИЧЧЯ
+А. Лоб*
+В. Скроні
+C. Зона брів
+СЕРЕДНЯ
+ТРЕТИНА ОБЛИЧЧЯ
+D. Моделювання носа*
+E. Аугментація малярної
+ та виличної зони
+F. Носогубні борозни
+НИЖНЯ
+ТРЕТИНА ОБЛИЧЧЯ
+G. Кути рота
+H. Зморшки маріонетки
+I. Підборіддя
+J. Лінія нижньої щелепи</t>
+  </si>
+  <si>
+    <t>4.</t>
+  </si>
+  <si>
+    <t>Зони та шари в яких застосовується препарат Ellanse</t>
+  </si>
+  <si>
+    <t>В яких зонах можна використовувати Ellanse?</t>
+  </si>
+  <si>
+    <t>Обличчя,шия,декольте</t>
+  </si>
+  <si>
+    <t>Обличчя,кисті</t>
+  </si>
+  <si>
+    <t>Тіло</t>
+  </si>
+  <si>
+    <t>Обличчя</t>
+  </si>
+  <si>
+    <t>Препарат Ellanse вводиться субдермально (В ПЖК -для збільшення субдермальних,поверхневих об'ємів)) або надперіостально (на кістку -для збільшення глибоких об'ємів)</t>
+  </si>
+  <si>
+    <t>В який шар потрібно вводити Ellanse?</t>
+  </si>
+  <si>
+    <t>субдермально та надперіостально</t>
+  </si>
+  <si>
+    <t>Тільки субдермально</t>
+  </si>
+  <si>
+    <t>Інтрадермально</t>
+  </si>
+  <si>
+    <t>Надперіостально</t>
+  </si>
+  <si>
+    <t>5.</t>
+  </si>
+  <si>
+    <t>Переваги  препарату Ellanse</t>
+  </si>
+  <si>
+    <t>Переваги для лікаря:1.Високий профіль безпеки:повна біодеградація
+ мікрочастинок PCL із часом 2.Прогнозований результат 3.Персоналізований підхід.
+Тривалість результату 18–24 місяців, залежно від препарату(Ellansé S або Ellansé M)
+ 4.Сертифікований у Європі (CЄ) та Україні  5.Підходить для всіх типів старіння
+обличчя (включаючи деформаційний) 6.Процедура не потребує знеболювання та
+розведення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Переваги препарату для пацієнта:1.Висока волюмізаційна здатність. Миттєва та помітна корекція зморшок і складок 2.Омолодження шляхом
+використання природного механізму і правильного колагеноутворення 3.Покращення якості шкіри 4.Короткий курс. Достатньо однієї процедури для
+досягнення бажаного ефекту на 18 або 24 міс.5.Відсутність реабілітаційного періоду. Процедура не обмежує соціальну активність.6.Відсутність
+фібротичних змін
+</t>
+  </si>
+  <si>
+    <t>Яка з наведених характеристик препарату Ellansé є однією з переваг для лікаря?</t>
+  </si>
+  <si>
+    <t>Потребує обов'язкового попереднього розведення перед введенням.</t>
+  </si>
+  <si>
+    <t>Високий профіль безпеки завдяки повній біодеградації мікрочастинок PCL.</t>
+  </si>
+  <si>
+    <t>Результат процедури зберігається не більше 6 місяців.</t>
+  </si>
+  <si>
+    <t>Препарат підходить лише для дрібнозморшкуватого типу старіння.</t>
+  </si>
+  <si>
+    <t>Яка комбінація переваг препарату Ellansé є найбільш вагомою для пацієнта, який веде активне соціальне життя і прагне природного омолодження?</t>
+  </si>
+  <si>
+    <t>Поступова корекція протягом року та необхідність тривалої реабілітації для закріплення ефекту.</t>
+  </si>
+  <si>
+    <t>Миттєва волюмізація, відсутність фібротичних змін та можливість не переривати соціальну активність.</t>
+  </si>
+  <si>
+    <t>Формування щільного фіброзу для утримання тканин та обов'язковий курс із 3-4 процедур.</t>
+  </si>
+  <si>
+    <t>Тимчасове обмеження міміки та використання зовнішніх стимуляторів колагену між процедурами.</t>
+  </si>
+  <si>
+    <t>Полімолочна кислота</t>
+  </si>
+  <si>
+    <t>Гідроксиапатит кальцію</t>
   </si>
   <si>
     <r>
@@ -256,189 +426,15 @@
         <charset val="204"/>
       </rPr>
       <t xml:space="preserve">
-- ГК дає об'єм на 6–12 міс, потім розсмоктується повністю
-- Ellansé: ефект 2–4 роки, замінюється власним колагеном пацієнта
-*Лінійка:* S (1 рік), M (2 роки), L (3 роки), E (4 роки)</t>
+</t>
     </r>
   </si>
   <si>
-    <t>Механізм дії та показання до застосування препарату Ellanse</t>
-  </si>
-  <si>
-    <t>Який механізм дії Ellanse?</t>
-  </si>
-  <si>
-    <t>1 крок: Миттєве відновлення об'єму,  2 крок: стимуляція синтезу власного колагену</t>
-  </si>
-  <si>
-    <t>1 крок:підготовка до синтезу колагену; 2 крок - синтез колагену; 3 крок -розпад колагену</t>
-  </si>
-  <si>
-    <t>1. Крок біоревіталізація; 2-біорепарація; 3- реструктуризація</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 крок відновлення об'єму; 2 крок-біодеградація </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Подвійна дія  Ellanse: 1.МИТТЄВЕ
-ВІДНОВЛЕННЯ ОБ’ЄМУ.Відбувається завдяки карбоксиметилцелюлозі
-Ellansé містить гладкі мікросфери,
-рівномірно розподілені в гелі-носії,
-які заповнюють ділянки шкіри,
-відновлюючи втрачений об’єм. КРОК 2: СТИМУЛЯЦІЯ
-СИНТЕЗУ ВЛАСНОГО
-КОЛАГЕНУ(довгострокова волюмізація-відбуваєтся завдяки полікапролактону):Протягом кількох місяців наявність
-гладких мікросфер посилює
-природний синтез колагену в
-шкірі. Мікросфери біодеградують
-із часом, а колагенові структури
-залишаються
+    <t xml:space="preserve">Мікросфери полікапролактону в Ellansé мають
+оптимальну біосумісність: гладеньку поверхню,
+сферичну форму, розмір 25–50 μm, повну
+біодеградацію з часом.
 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ellanse показаний 1.Чоловікам та  жінкам старше 18 років
-2.З будь-яким типом старіння
-3.Які хочуть поступових покращень з довгостроковим результатом:
--Untouched face
--Відновлення втрачених об’ємів
--Ліфтингу
--Зменшення асиметрії
--Чіткого контуру та овалу  обличчя
--Покращення пружності та еластичності шкіри
-</t>
-  </si>
-  <si>
-    <t>Що НЕ являється показанням для проведення процедури Ellanse</t>
-  </si>
-  <si>
-    <t>Untouched face</t>
-  </si>
-  <si>
-    <t>Втрата об'єму</t>
-  </si>
-  <si>
-    <t>Зниження пружності шкіри</t>
-  </si>
-  <si>
-    <t>Гіперпігментація</t>
-  </si>
-  <si>
-    <t>Механізм дії та показання до застосування препарату Ellanse,зонивведення</t>
-  </si>
-  <si>
-    <t>Ellanse використовується тільки для корекції наступних зон обличчя:ВЕРХНЯ
-ТРЕТИНА ОБЛИЧЧЯ
-А. Лоб*
-В. Скроні
-C. Зона брів
-СЕРЕДНЯ
-ТРЕТИНА ОБЛИЧЧЯ
-D. Моделювання носа*
-E. Аугментація малярної
- та виличної зони
-F. Носогубні борозни
-НИЖНЯ
-ТРЕТИНА ОБЛИЧЧЯ
-G. Кути рота
-H. Зморшки маріонетки
-I. Підборіддя
-J. Лінія нижньої щелепи</t>
-  </si>
-  <si>
-    <t>4.</t>
-  </si>
-  <si>
-    <t>Зони та шари в яких застосовується препарат Ellanse</t>
-  </si>
-  <si>
-    <t>В яких зонах можна використовувати Ellanse?</t>
-  </si>
-  <si>
-    <t>Обличчя,шия,декольте</t>
-  </si>
-  <si>
-    <t>Обличчя,кисті</t>
-  </si>
-  <si>
-    <t>Тіло</t>
-  </si>
-  <si>
-    <t>Обличчя</t>
-  </si>
-  <si>
-    <t>Препарат Ellanse вводиться субдермально (В ПЖК -для збільшення субдермальних,поверхневих об'ємів)) або надперіостально (на кістку -для збільшення глибоких об'ємів)</t>
-  </si>
-  <si>
-    <t>В який шар потрібно вводити Ellanse?</t>
-  </si>
-  <si>
-    <t>субдермально та надперіостально</t>
-  </si>
-  <si>
-    <t>Тільки субдермально</t>
-  </si>
-  <si>
-    <t>Інтрадермально</t>
-  </si>
-  <si>
-    <t>Надперіостально</t>
-  </si>
-  <si>
-    <t>5.</t>
-  </si>
-  <si>
-    <t>Переваги  препарату Ellanse</t>
-  </si>
-  <si>
-    <t>Переваги для лікаря:1.Високий профіль безпеки:повна біодеградація
- мікрочастинок PCL із часом 2.Прогнозований результат 3.Персоналізований підхід.
-Тривалість результату 18–24 місяців, залежно від препарату(Ellansé S або Ellansé M)
- 4.Сертифікований у Європі (CЄ) та Україні  5.Підходить для всіх типів старіння
-обличчя (включаючи деформаційний) 6.Процедура не потребує знеболювання та
-розведення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Переваги препарату для пацієнта:1.Висока волюмізаційна здатність. Миттєва та помітна корекція зморшок і складок 2.Омолодження шляхом
-використання природного механізму і правильного колагеноутворення 3.Покращення якості шкіри 4.Короткий курс. Достатньо однієї процедури для
-досягнення бажаного ефекту на 18 або 24 міс.5.Відсутність реабілітаційного періоду. Процедура не обмежує соціальну активність.6.Відсутність
-фібротичних змін
-</t>
-  </si>
-  <si>
-    <t>Яка з наведених характеристик препарату Ellansé є однією з переваг для лікаря?</t>
-  </si>
-  <si>
-    <t>Потребує обов'язкового попереднього розведення перед введенням.</t>
-  </si>
-  <si>
-    <t>Високий профіль безпеки завдяки повній біодеградації мікрочастинок PCL.</t>
-  </si>
-  <si>
-    <t>Результат процедури зберігається не більше 6 місяців.</t>
-  </si>
-  <si>
-    <t>Препарат підходить лише для дрібнозморшкуватого типу старіння.</t>
-  </si>
-  <si>
-    <t>Яка комбінація переваг препарату Ellansé є найбільш вагомою для пацієнта, який веде активне соціальне життя і прагне природного омолодження?</t>
-  </si>
-  <si>
-    <t>Поступова корекція протягом року та необхідність тривалої реабілітації для закріплення ефекту.</t>
-  </si>
-  <si>
-    <t>Миттєва волюмізація, відсутність фібротичних змін та можливість не переривати соціальну активність.</t>
-  </si>
-  <si>
-    <t>Формування щільного фіброзу для утримання тканин та обов'язковий курс із 3-4 процедур.</t>
-  </si>
-  <si>
-    <t>Тимчасове обмеження міміки та використання зовнішніх стимуляторів колагену між процедурами.</t>
-  </si>
-  <si>
-    <t>Полімолочна кислота</t>
-  </si>
-  <si>
-    <t>Гідроксиапатит кальцію</t>
   </si>
 </sst>
 </file>
@@ -1576,15 +1572,15 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="386.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12">
         <v>1</v>
       </c>
       <c r="B2" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="14" t="s">
-        <v>64</v>
+      <c r="C2" s="12" t="s">
+        <v>107</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>30</v>
@@ -1596,10 +1592,10 @@
         <v>32</v>
       </c>
       <c r="G2" s="14" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I2" s="12">
         <v>2</v>
@@ -1663,15 +1659,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="251.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="13">
         <v>2</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>51</v>
+      <c r="C5" s="13" t="s">
+        <v>108</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>46</v>
@@ -1700,22 +1696,22 @@
         <v>45</v>
       </c>
       <c r="C6" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="E6" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="F6" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="G6" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="H6" s="15" t="s">
         <v>56</v>
-      </c>
-      <c r="H6" s="15" t="s">
-        <v>57</v>
       </c>
       <c r="I6" s="13">
         <v>3</v>
@@ -1729,22 +1725,22 @@
         <v>45</v>
       </c>
       <c r="C7" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="17" t="s">
         <v>59</v>
       </c>
-      <c r="D7" t="s">
-        <v>58</v>
-      </c>
-      <c r="E7" s="17" t="s">
+      <c r="F7" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="G7" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="G7" s="17" t="s">
+      <c r="H7" s="17" t="s">
         <v>62</v>
-      </c>
-      <c r="H7" s="17" t="s">
-        <v>63</v>
       </c>
       <c r="I7" s="16">
         <v>2</v>
@@ -1755,25 +1751,25 @@
         <v>3</v>
       </c>
       <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E8" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="F8" s="17" t="s">
         <v>66</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="G8" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="H8" s="17" t="s">
         <v>68</v>
-      </c>
-      <c r="G8" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>70</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -1784,25 +1780,25 @@
         <v>3</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C9" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="D9" t="s">
+      <c r="F9" s="17" t="s">
         <v>73</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="G9" s="17" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="H9" s="17" t="s">
         <v>75</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="H9" s="17" t="s">
-        <v>77</v>
       </c>
       <c r="I9">
         <v>4</v>
@@ -1810,28 +1806,28 @@
     </row>
     <row r="10" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" t="s">
         <v>80</v>
       </c>
-      <c r="B10" t="s">
+      <c r="E10" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="F10" s="17" t="s">
         <v>82</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="G10" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="H10" s="17" t="s">
         <v>84</v>
-      </c>
-      <c r="G10" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="H10" s="17" t="s">
-        <v>86</v>
       </c>
       <c r="I10">
         <v>4</v>
@@ -1839,28 +1835,28 @@
     </row>
     <row r="11" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C11" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="D11" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="D11" t="s">
+      <c r="F11" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="G11" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="H11" s="17" t="s">
         <v>90</v>
-      </c>
-      <c r="G11" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="H11" s="17" t="s">
-        <v>92</v>
       </c>
       <c r="I11">
         <v>1</v>
@@ -1868,28 +1864,28 @@
     </row>
     <row r="12" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="B12" t="s">
-        <v>94</v>
-      </c>
-      <c r="C12" s="18" t="s">
+      <c r="D12" t="s">
         <v>95</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="G12" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="H12" s="17" t="s">
         <v>99</v>
-      </c>
-      <c r="G12" s="17" t="s">
-        <v>100</v>
-      </c>
-      <c r="H12" s="17" t="s">
-        <v>101</v>
       </c>
       <c r="I12">
         <v>2</v>
@@ -1897,25 +1893,25 @@
     </row>
     <row r="13" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
+        <v>92</v>
+      </c>
+      <c r="C13" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="C13" s="18" t="s">
-        <v>96</v>
-      </c>
       <c r="D13" t="s">
+        <v>100</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="F13" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="G13" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="H13" s="17" t="s">
         <v>104</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="H13" s="17" t="s">
-        <v>106</v>
       </c>
       <c r="I13">
         <v>2</v>

</xml_diff>